<commit_message>
Add unit testing and threat analysis results
- Document unit testing results for Secure Boot firmware integrity validation and A/B FOTA.
- Include threat analysis results and identified security considerations.
- Consolidate test outcomes and threat findings for project documentation and traceability.
</commit_message>
<xml_diff>
--- a/Validation/STM32_Secure_Boot_Validation.xlsx
+++ b/Validation/STM32_Secure_Boot_Validation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Manisha Daigavhane\software\workspace\Github_Repositories\STM32-Project-05-Secure-Boot\Validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64FBEA09-C762-4A77-A6F8-9AA41C8E205A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37CF08C-6C07-4AD4-9A06-167E9FC99970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="634">
   <si>
     <t>Field</t>
   </si>
@@ -6095,6 +6095,104 @@
   </si>
   <si>
     <t xml:space="preserve">Total </t>
+  </si>
+  <si>
+    <t>MEM-014</t>
+  </si>
+  <si>
+    <t>Staging and Destination Programming Boundary Validation</t>
+  </si>
+  <si>
+    <t>Firmware programming shall reject image sizes exceeding the permitted capacity of the staging area or destination slot before writing to flash.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Verify the 64 KB staging limit and 128 KB Slot A/Slot B limits in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FlashStorage_ProgramImage()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Updated boundary checks are present. Use a mocked or controlled flash-programming interface.</t>
+  </si>
+  <si>
+    <t>HR-03 verification. Account for 32-bit word rounding.</t>
+  </si>
+  <si>
+    <t>MEM-014_Staging_Boundary_Validation</t>
+  </si>
+  <si>
+    <t>FOTA-VAL-013</t>
+  </si>
+  <si>
+    <t>Flash Erase/Program Failure Handling</t>
+  </si>
+  <si>
+    <t>Flash erase, programming, and metadata commit operations shall detect failures and propagate errors without reporting a failed update as successful.</t>
+  </si>
+  <si>
+    <t>Verify flash-operation error handling and metadata commit failure behavior.</t>
+  </si>
+  <si>
+    <t>Updated flash unlock checks are present. Use mocked HAL functions or controlled fault injection.</t>
+  </si>
+  <si>
+    <t>Each failure is reported. Failed operations are not reported as successful, promotion does not advance incorrectly, and metadata is accepted only after required verification and commit checks succeed.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">HR-05 verification. Test metadata failures through </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Metadata_WriteRecord()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>FOTA-VAL-013Flash_Erase_Program_Failure_Handling</t>
+  </si>
+  <si>
+    <t>1. Test 64 KB + 1 byte staging write. 
+2. Verify rejected requests do not invoke flash programming.</t>
+  </si>
+  <si>
+    <t>Writes within staging region's capacity pass the boundary check. Oversized writes are rejected before flash programming.</t>
+  </si>
+  <si>
+    <t>Oversized writes are rejected before flash programming.</t>
+  </si>
+  <si>
+    <t>1. Simulate flash unlock failure. 2. Check returned status and update-state handling.</t>
   </si>
 </sst>
 </file>
@@ -6208,9 +6306,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -6218,6 +6313,9 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6807,12 +6905,12 @@
       <c r="B9" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6825,7 +6923,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD55151-40F8-416C-98E3-A78CDE29E48B}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="13.77734375" customWidth="1"/>
@@ -7328,6 +7426,41 @@
       </c>
       <c r="K14" s="6" t="s">
         <v>222</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" s="2" customFormat="1" ht="100.8">
+      <c r="A15" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>620</v>
       </c>
     </row>
   </sheetData>
@@ -7712,7 +7845,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05E5142-AEE3-4F3C-9EE7-B4A55C2203BE}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.6640625" customWidth="1"/>
@@ -8180,6 +8313,41 @@
       </c>
       <c r="K13" s="2" t="s">
         <v>390</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="129.6">
+      <c r="A14" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>627</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>628</v>
       </c>
     </row>
   </sheetData>
@@ -9059,7 +9227,7 @@
       <c r="D2" s="9">
         <v>0</v>
       </c>
-      <c r="E2" s="17">
+      <c r="E2" s="16">
         <v>1</v>
       </c>
     </row>
@@ -9068,15 +9236,15 @@
         <v>298</v>
       </c>
       <c r="B3" s="9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" s="9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" s="9">
         <v>0</v>
       </c>
-      <c r="E3" s="17">
+      <c r="E3" s="16">
         <v>1</v>
       </c>
     </row>
@@ -9093,7 +9261,7 @@
       <c r="D4" s="9">
         <v>0</v>
       </c>
-      <c r="E4" s="17">
+      <c r="E4" s="16">
         <v>1</v>
       </c>
     </row>
@@ -9102,15 +9270,15 @@
         <v>318</v>
       </c>
       <c r="B5" s="9">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" s="9">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="9">
         <v>0</v>
       </c>
-      <c r="E5" s="17">
+      <c r="E5" s="16">
         <v>1</v>
       </c>
     </row>
@@ -9127,26 +9295,26 @@
       <c r="D6" s="9">
         <v>0</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="15" t="s">
         <v>614</v>
       </c>
       <c r="B7" s="10">
         <f>B2+B3+B4+B5+B6</f>
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C7" s="10">
         <f>SUM(C2:C6)</f>
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D7" s="9">
         <v>0</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="17">
         <v>1</v>
       </c>
     </row>

</xml_diff>